<commit_message>
Updated IDN_grids_kan model - 2026-04-27 18:25
</commit_message>
<xml_diff>
--- a/VerveStacks_IDN_grids_kan/Sets-vervestacks.xlsx
+++ b/VerveStacks_IDN_grids_kan/Sets-vervestacks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr updateLinks="never" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_IDN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{34164E1E-A9A5-476B-874C-EFD844CE8621}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{45E135DA-36D0-4830-B30A-D4FD32B866F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1124" uniqueCount="606">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1132" uniqueCount="610">
   <si>
     <t>~TFM_Psets</t>
   </si>
@@ -349,1513 +349,1525 @@
     <t>t_pos_andor</t>
   </si>
   <si>
-    <t>p_w159940153</t>
-  </si>
-  <si>
-    <t>e_w159940153*</t>
+    <t>p_w159940153-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w159940153-500_IDN*</t>
   </si>
   <si>
     <t>OR</t>
   </si>
   <si>
-    <t>p_w161960924</t>
-  </si>
-  <si>
-    <t>e_w161960924*</t>
-  </si>
-  <si>
-    <t>p_w161960933</t>
-  </si>
-  <si>
-    <t>e_w161960933*</t>
-  </si>
-  <si>
-    <t>p_w161965853</t>
-  </si>
-  <si>
-    <t>e_w161965853*</t>
-  </si>
-  <si>
-    <t>p_w166633831</t>
-  </si>
-  <si>
-    <t>e_w166633831*</t>
-  </si>
-  <si>
-    <t>p_w169444592</t>
-  </si>
-  <si>
-    <t>e_w169444592*</t>
-  </si>
-  <si>
-    <t>p_w261185002</t>
-  </si>
-  <si>
-    <t>e_w261185002*</t>
-  </si>
-  <si>
-    <t>p_w264410236</t>
-  </si>
-  <si>
-    <t>e_w264410236*</t>
-  </si>
-  <si>
-    <t>p_w264550744</t>
-  </si>
-  <si>
-    <t>e_w264550744*</t>
-  </si>
-  <si>
-    <t>p_w265318414</t>
-  </si>
-  <si>
-    <t>e_w265318414*</t>
-  </si>
-  <si>
-    <t>p_w265568001</t>
-  </si>
-  <si>
-    <t>e_w265568001*</t>
-  </si>
-  <si>
-    <t>p_w267626657</t>
-  </si>
-  <si>
-    <t>e_w267626657*</t>
-  </si>
-  <si>
-    <t>p_w271376037</t>
-  </si>
-  <si>
-    <t>e_w271376037*</t>
-  </si>
-  <si>
-    <t>p_w310695690</t>
-  </si>
-  <si>
-    <t>e_w310695690*</t>
-  </si>
-  <si>
-    <t>p_w310958602</t>
-  </si>
-  <si>
-    <t>e_w310958602*</t>
-  </si>
-  <si>
-    <t>p_w314452486</t>
-  </si>
-  <si>
-    <t>e_w314452486*</t>
-  </si>
-  <si>
-    <t>p_w337039411</t>
-  </si>
-  <si>
-    <t>e_w337039411*</t>
-  </si>
-  <si>
-    <t>p_w340205049</t>
-  </si>
-  <si>
-    <t>e_w340205049*</t>
-  </si>
-  <si>
-    <t>p_w340978681</t>
-  </si>
-  <si>
-    <t>e_w340978681*</t>
-  </si>
-  <si>
-    <t>p_w398909640</t>
-  </si>
-  <si>
-    <t>e_w398909640*</t>
-  </si>
-  <si>
-    <t>p_w399038181</t>
-  </si>
-  <si>
-    <t>e_w399038181*</t>
-  </si>
-  <si>
-    <t>p_w399100034</t>
-  </si>
-  <si>
-    <t>e_w399100034*</t>
-  </si>
-  <si>
-    <t>p_w399100035</t>
-  </si>
-  <si>
-    <t>e_w399100035*</t>
-  </si>
-  <si>
-    <t>p_w469888049</t>
-  </si>
-  <si>
-    <t>e_w469888049*</t>
-  </si>
-  <si>
-    <t>p_w527900241</t>
-  </si>
-  <si>
-    <t>e_w527900241*</t>
-  </si>
-  <si>
-    <t>p_w528189342</t>
-  </si>
-  <si>
-    <t>e_w528189342*</t>
-  </si>
-  <si>
-    <t>p_w544403426</t>
-  </si>
-  <si>
-    <t>e_w544403426*</t>
-  </si>
-  <si>
-    <t>p_w544403431</t>
-  </si>
-  <si>
-    <t>e_w544403431*</t>
-  </si>
-  <si>
-    <t>p_w562061281</t>
-  </si>
-  <si>
-    <t>e_w562061281*</t>
-  </si>
-  <si>
-    <t>p_w604684007</t>
-  </si>
-  <si>
-    <t>e_w604684007*</t>
-  </si>
-  <si>
-    <t>p_w610198177</t>
-  </si>
-  <si>
-    <t>e_w610198177*</t>
-  </si>
-  <si>
-    <t>p_w614955990</t>
-  </si>
-  <si>
-    <t>e_w614955990*</t>
-  </si>
-  <si>
-    <t>p_w614955993</t>
-  </si>
-  <si>
-    <t>e_w614955993*</t>
-  </si>
-  <si>
-    <t>p_w615581232</t>
-  </si>
-  <si>
-    <t>e_w615581232*</t>
-  </si>
-  <si>
-    <t>p_w615581242</t>
-  </si>
-  <si>
-    <t>e_w615581242*</t>
-  </si>
-  <si>
-    <t>p_w615581270</t>
-  </si>
-  <si>
-    <t>e_w615581270*</t>
-  </si>
-  <si>
-    <t>p_w629512849</t>
-  </si>
-  <si>
-    <t>e_w629512849*</t>
-  </si>
-  <si>
-    <t>p_w662591948</t>
-  </si>
-  <si>
-    <t>e_w662591948*</t>
-  </si>
-  <si>
-    <t>p_w689263666</t>
-  </si>
-  <si>
-    <t>e_w689263666*</t>
-  </si>
-  <si>
-    <t>p_w721674155</t>
-  </si>
-  <si>
-    <t>e_w721674155*</t>
-  </si>
-  <si>
-    <t>p_w721685825</t>
-  </si>
-  <si>
-    <t>e_w721685825*</t>
-  </si>
-  <si>
-    <t>p_w736595653</t>
-  </si>
-  <si>
-    <t>e_w736595653*</t>
-  </si>
-  <si>
-    <t>p_w753733608</t>
-  </si>
-  <si>
-    <t>e_w753733608*</t>
-  </si>
-  <si>
-    <t>p_w754073846</t>
-  </si>
-  <si>
-    <t>e_w754073846*</t>
-  </si>
-  <si>
-    <t>p_w754096394</t>
-  </si>
-  <si>
-    <t>e_w754096394*</t>
-  </si>
-  <si>
-    <t>p_w754178666</t>
-  </si>
-  <si>
-    <t>e_w754178666*</t>
-  </si>
-  <si>
-    <t>p_w754178667</t>
-  </si>
-  <si>
-    <t>e_w754178667*</t>
-  </si>
-  <si>
-    <t>p_w759130125</t>
-  </si>
-  <si>
-    <t>e_w759130125*</t>
-  </si>
-  <si>
-    <t>p_w769617021</t>
-  </si>
-  <si>
-    <t>e_w769617021*</t>
-  </si>
-  <si>
-    <t>p_w841499143</t>
-  </si>
-  <si>
-    <t>e_w841499143*</t>
-  </si>
-  <si>
-    <t>p_w926254403</t>
-  </si>
-  <si>
-    <t>e_w926254403*</t>
-  </si>
-  <si>
-    <t>p_w928220391</t>
-  </si>
-  <si>
-    <t>e_w928220391*</t>
-  </si>
-  <si>
-    <t>p_w928928133</t>
-  </si>
-  <si>
-    <t>e_w928928133*</t>
-  </si>
-  <si>
-    <t>p_w930719092</t>
-  </si>
-  <si>
-    <t>e_w930719092*</t>
-  </si>
-  <si>
-    <t>p_w931931121</t>
-  </si>
-  <si>
-    <t>e_w931931121*</t>
-  </si>
-  <si>
-    <t>p_w931931133</t>
-  </si>
-  <si>
-    <t>e_w931931133*</t>
-  </si>
-  <si>
-    <t>p_w939542521</t>
-  </si>
-  <si>
-    <t>e_w939542521*</t>
-  </si>
-  <si>
-    <t>p_w943539373</t>
-  </si>
-  <si>
-    <t>e_w943539373*</t>
-  </si>
-  <si>
-    <t>p_w946191122</t>
-  </si>
-  <si>
-    <t>e_w946191122*</t>
-  </si>
-  <si>
-    <t>p_w960747902</t>
-  </si>
-  <si>
-    <t>e_w960747902*</t>
-  </si>
-  <si>
-    <t>p_w960747936</t>
-  </si>
-  <si>
-    <t>e_w960747936*</t>
-  </si>
-  <si>
-    <t>p_w966209515</t>
-  </si>
-  <si>
-    <t>e_w966209515*</t>
-  </si>
-  <si>
-    <t>p_w1013653012</t>
-  </si>
-  <si>
-    <t>e_w1013653012*</t>
-  </si>
-  <si>
-    <t>p_w1186182648</t>
-  </si>
-  <si>
-    <t>e_w1186182648*</t>
-  </si>
-  <si>
-    <t>p_w1193553154</t>
-  </si>
-  <si>
-    <t>e_w1193553154*</t>
-  </si>
-  <si>
-    <t>p_w1308433899</t>
-  </si>
-  <si>
-    <t>e_w1308433899*</t>
-  </si>
-  <si>
-    <t>p_w1312287191</t>
-  </si>
-  <si>
-    <t>e_w1312287191*</t>
-  </si>
-  <si>
-    <t>p_w1316786278</t>
-  </si>
-  <si>
-    <t>e_w1316786278*</t>
-  </si>
-  <si>
-    <t>p_w1316876158</t>
-  </si>
-  <si>
-    <t>e_w1316876158*</t>
-  </si>
-  <si>
-    <t>p_ID36</t>
-  </si>
-  <si>
-    <t>e_ID36*</t>
-  </si>
-  <si>
-    <t>p_ID11</t>
-  </si>
-  <si>
-    <t>e_ID11*</t>
-  </si>
-  <si>
-    <t>p_ID26</t>
-  </si>
-  <si>
-    <t>e_ID26*</t>
-  </si>
-  <si>
-    <t>p_ID13</t>
-  </si>
-  <si>
-    <t>e_ID13*</t>
-  </si>
-  <si>
-    <t>p_ID22</t>
-  </si>
-  <si>
-    <t>e_ID22*</t>
-  </si>
-  <si>
-    <t>p_ID38</t>
-  </si>
-  <si>
-    <t>e_ID38*</t>
-  </si>
-  <si>
-    <t>p_ID34</t>
-  </si>
-  <si>
-    <t>e_ID34*</t>
-  </si>
-  <si>
-    <t>p_ID1</t>
-  </si>
-  <si>
-    <t>e_ID1*</t>
-  </si>
-  <si>
-    <t>p_ID31</t>
-  </si>
-  <si>
-    <t>e_ID31*</t>
-  </si>
-  <si>
-    <t>p_ID4</t>
-  </si>
-  <si>
-    <t>e_ID4*</t>
-  </si>
-  <si>
-    <t>p_ID5</t>
-  </si>
-  <si>
-    <t>e_ID5*</t>
-  </si>
-  <si>
-    <t>p_ID6</t>
-  </si>
-  <si>
-    <t>e_ID6*</t>
-  </si>
-  <si>
-    <t>p_ID7</t>
-  </si>
-  <si>
-    <t>e_ID7*</t>
-  </si>
-  <si>
-    <t>p_ID12</t>
-  </si>
-  <si>
-    <t>e_ID12*</t>
-  </si>
-  <si>
-    <t>p_ID28</t>
-  </si>
-  <si>
-    <t>e_ID28*</t>
-  </si>
-  <si>
-    <t>p_ID27</t>
-  </si>
-  <si>
-    <t>e_ID27*</t>
-  </si>
-  <si>
-    <t>p_ID25</t>
-  </si>
-  <si>
-    <t>e_ID25*</t>
-  </si>
-  <si>
-    <t>p_ID33</t>
-  </si>
-  <si>
-    <t>e_ID33*</t>
-  </si>
-  <si>
-    <t>p_ID37</t>
-  </si>
-  <si>
-    <t>e_ID37*</t>
-  </si>
-  <si>
-    <t>p_ID10</t>
-  </si>
-  <si>
-    <t>e_ID10*</t>
-  </si>
-  <si>
-    <t>p_ID16</t>
-  </si>
-  <si>
-    <t>e_ID16*</t>
-  </si>
-  <si>
-    <t>p_ID8</t>
-  </si>
-  <si>
-    <t>e_ID8*</t>
-  </si>
-  <si>
-    <t>p_ID14</t>
-  </si>
-  <si>
-    <t>e_ID14*</t>
-  </si>
-  <si>
-    <t>p_ID18</t>
-  </si>
-  <si>
-    <t>e_ID18*</t>
-  </si>
-  <si>
-    <t>p_ID21</t>
-  </si>
-  <si>
-    <t>e_ID21*</t>
-  </si>
-  <si>
-    <t>p_ID20</t>
-  </si>
-  <si>
-    <t>e_ID20*</t>
-  </si>
-  <si>
-    <t>p_ID24</t>
-  </si>
-  <si>
-    <t>e_ID24*</t>
-  </si>
-  <si>
-    <t>p_ID2</t>
-  </si>
-  <si>
-    <t>e_ID2*</t>
-  </si>
-  <si>
-    <t>p_ID9</t>
-  </si>
-  <si>
-    <t>e_ID9*</t>
-  </si>
-  <si>
-    <t>p_ID30</t>
-  </si>
-  <si>
-    <t>e_ID30*</t>
-  </si>
-  <si>
-    <t>p_ID3</t>
-  </si>
-  <si>
-    <t>e_ID3*</t>
-  </si>
-  <si>
-    <t>p_ID23</t>
-  </si>
-  <si>
-    <t>e_ID23*</t>
-  </si>
-  <si>
-    <t>p_ID29</t>
-  </si>
-  <si>
-    <t>e_ID29*</t>
-  </si>
-  <si>
-    <t>p_ID35</t>
-  </si>
-  <si>
-    <t>e_ID35*</t>
-  </si>
-  <si>
-    <t>p_ID19</t>
-  </si>
-  <si>
-    <t>e_ID19*</t>
-  </si>
-  <si>
-    <t>p_ID17</t>
-  </si>
-  <si>
-    <t>e_ID17*</t>
-  </si>
-  <si>
-    <t>p_ID15</t>
-  </si>
-  <si>
-    <t>e_ID15*</t>
-  </si>
-  <si>
-    <t>rez_spv_001</t>
-  </si>
-  <si>
-    <t>elc_spv_001</t>
-  </si>
-  <si>
-    <t>rez_spv_002</t>
-  </si>
-  <si>
-    <t>elc_spv_002</t>
-  </si>
-  <si>
-    <t>rez_spv_003</t>
-  </si>
-  <si>
-    <t>elc_spv_003</t>
-  </si>
-  <si>
-    <t>rez_spv_004</t>
-  </si>
-  <si>
-    <t>elc_spv_004</t>
-  </si>
-  <si>
-    <t>rez_spv_005</t>
-  </si>
-  <si>
-    <t>elc_spv_005</t>
-  </si>
-  <si>
-    <t>rez_spv_006</t>
-  </si>
-  <si>
-    <t>elc_spv_006</t>
-  </si>
-  <si>
-    <t>rez_spv_007</t>
-  </si>
-  <si>
-    <t>elc_spv_007</t>
-  </si>
-  <si>
-    <t>rez_spv_008</t>
-  </si>
-  <si>
-    <t>elc_spv_008</t>
-  </si>
-  <si>
-    <t>rez_spv_009</t>
-  </si>
-  <si>
-    <t>elc_spv_009</t>
-  </si>
-  <si>
-    <t>rez_spv_010</t>
-  </si>
-  <si>
-    <t>elc_spv_010</t>
-  </si>
-  <si>
-    <t>rez_spv_011</t>
-  </si>
-  <si>
-    <t>elc_spv_011</t>
-  </si>
-  <si>
-    <t>rez_spv_012</t>
-  </si>
-  <si>
-    <t>elc_spv_012</t>
-  </si>
-  <si>
-    <t>rez_spv_013</t>
-  </si>
-  <si>
-    <t>elc_spv_013</t>
-  </si>
-  <si>
-    <t>rez_spv_014</t>
-  </si>
-  <si>
-    <t>elc_spv_014</t>
-  </si>
-  <si>
-    <t>rez_spv_015</t>
-  </si>
-  <si>
-    <t>elc_spv_015</t>
-  </si>
-  <si>
-    <t>rez_spv_016</t>
-  </si>
-  <si>
-    <t>elc_spv_016</t>
-  </si>
-  <si>
-    <t>rez_spv_017</t>
-  </si>
-  <si>
-    <t>elc_spv_017</t>
-  </si>
-  <si>
-    <t>rez_spv_018</t>
-  </si>
-  <si>
-    <t>elc_spv_018</t>
-  </si>
-  <si>
-    <t>rez_spv_019</t>
-  </si>
-  <si>
-    <t>elc_spv_019</t>
-  </si>
-  <si>
-    <t>rez_spv_020</t>
-  </si>
-  <si>
-    <t>elc_spv_020</t>
-  </si>
-  <si>
-    <t>rez_spv_021</t>
-  </si>
-  <si>
-    <t>elc_spv_021</t>
-  </si>
-  <si>
-    <t>rez_spv_022</t>
-  </si>
-  <si>
-    <t>elc_spv_022</t>
-  </si>
-  <si>
-    <t>rez_spv_023</t>
-  </si>
-  <si>
-    <t>elc_spv_023</t>
-  </si>
-  <si>
-    <t>rez_spv_024</t>
-  </si>
-  <si>
-    <t>elc_spv_024</t>
-  </si>
-  <si>
-    <t>rez_spv_025</t>
-  </si>
-  <si>
-    <t>elc_spv_025</t>
-  </si>
-  <si>
-    <t>rez_spv_026</t>
-  </si>
-  <si>
-    <t>elc_spv_026</t>
-  </si>
-  <si>
-    <t>rez_spv_027</t>
-  </si>
-  <si>
-    <t>elc_spv_027</t>
-  </si>
-  <si>
-    <t>rez_spv_028</t>
-  </si>
-  <si>
-    <t>elc_spv_028</t>
-  </si>
-  <si>
-    <t>rez_spv_029</t>
-  </si>
-  <si>
-    <t>elc_spv_029</t>
-  </si>
-  <si>
-    <t>rez_spv_030</t>
-  </si>
-  <si>
-    <t>elc_spv_030</t>
-  </si>
-  <si>
-    <t>rez_spv_031</t>
-  </si>
-  <si>
-    <t>elc_spv_031</t>
-  </si>
-  <si>
-    <t>rez_spv_032</t>
-  </si>
-  <si>
-    <t>elc_spv_032</t>
-  </si>
-  <si>
-    <t>rez_spv_033</t>
-  </si>
-  <si>
-    <t>elc_spv_033</t>
-  </si>
-  <si>
-    <t>rez_spv_034</t>
-  </si>
-  <si>
-    <t>elc_spv_034</t>
-  </si>
-  <si>
-    <t>rez_spv_035</t>
-  </si>
-  <si>
-    <t>elc_spv_035</t>
-  </si>
-  <si>
-    <t>rez_spv_036</t>
-  </si>
-  <si>
-    <t>elc_spv_036</t>
-  </si>
-  <si>
-    <t>rez_spv_037</t>
-  </si>
-  <si>
-    <t>elc_spv_037</t>
-  </si>
-  <si>
-    <t>rez_spv_038</t>
-  </si>
-  <si>
-    <t>elc_spv_038</t>
-  </si>
-  <si>
-    <t>rez_spv_039</t>
-  </si>
-  <si>
-    <t>elc_spv_039</t>
-  </si>
-  <si>
-    <t>rez_spv_040</t>
-  </si>
-  <si>
-    <t>elc_spv_040</t>
-  </si>
-  <si>
-    <t>rez_spv_041</t>
-  </si>
-  <si>
-    <t>elc_spv_041</t>
-  </si>
-  <si>
-    <t>rez_spv_042</t>
-  </si>
-  <si>
-    <t>elc_spv_042</t>
-  </si>
-  <si>
-    <t>rez_spv_043</t>
-  </si>
-  <si>
-    <t>elc_spv_043</t>
-  </si>
-  <si>
-    <t>rez_spv_044</t>
-  </si>
-  <si>
-    <t>elc_spv_044</t>
-  </si>
-  <si>
-    <t>rez_spv_045</t>
-  </si>
-  <si>
-    <t>elc_spv_045</t>
-  </si>
-  <si>
-    <t>rez_spv_046</t>
-  </si>
-  <si>
-    <t>elc_spv_046</t>
-  </si>
-  <si>
-    <t>rez_spv_047</t>
-  </si>
-  <si>
-    <t>elc_spv_047</t>
-  </si>
-  <si>
-    <t>rez_spv_048</t>
-  </si>
-  <si>
-    <t>elc_spv_048</t>
-  </si>
-  <si>
-    <t>rez_spv_049</t>
-  </si>
-  <si>
-    <t>elc_spv_049</t>
-  </si>
-  <si>
-    <t>rez_spv_050</t>
-  </si>
-  <si>
-    <t>elc_spv_050</t>
-  </si>
-  <si>
-    <t>rez_spv_051</t>
-  </si>
-  <si>
-    <t>elc_spv_051</t>
-  </si>
-  <si>
-    <t>rez_spv_052</t>
-  </si>
-  <si>
-    <t>elc_spv_052</t>
-  </si>
-  <si>
-    <t>rez_spv_053</t>
-  </si>
-  <si>
-    <t>elc_spv_053</t>
-  </si>
-  <si>
-    <t>rez_spv_054</t>
-  </si>
-  <si>
-    <t>elc_spv_054</t>
-  </si>
-  <si>
-    <t>rez_spv_055</t>
-  </si>
-  <si>
-    <t>elc_spv_055</t>
-  </si>
-  <si>
-    <t>rez_spv_056</t>
-  </si>
-  <si>
-    <t>elc_spv_056</t>
-  </si>
-  <si>
-    <t>rez_spv_057</t>
-  </si>
-  <si>
-    <t>elc_spv_057</t>
-  </si>
-  <si>
-    <t>rez_spv_058</t>
-  </si>
-  <si>
-    <t>elc_spv_058</t>
-  </si>
-  <si>
-    <t>rez_spv_059</t>
-  </si>
-  <si>
-    <t>elc_spv_059</t>
-  </si>
-  <si>
-    <t>rez_spv_060</t>
-  </si>
-  <si>
-    <t>elc_spv_060</t>
-  </si>
-  <si>
-    <t>rez_spv_061</t>
-  </si>
-  <si>
-    <t>elc_spv_061</t>
-  </si>
-  <si>
-    <t>rez_spv_062</t>
-  </si>
-  <si>
-    <t>elc_spv_062</t>
-  </si>
-  <si>
-    <t>rez_spv_063</t>
-  </si>
-  <si>
-    <t>elc_spv_063</t>
-  </si>
-  <si>
-    <t>rez_spv_064</t>
-  </si>
-  <si>
-    <t>elc_spv_064</t>
-  </si>
-  <si>
-    <t>rez_spv_065</t>
-  </si>
-  <si>
-    <t>elc_spv_065</t>
-  </si>
-  <si>
-    <t>rez_spv_066</t>
-  </si>
-  <si>
-    <t>elc_spv_066</t>
-  </si>
-  <si>
-    <t>rez_spv_067</t>
-  </si>
-  <si>
-    <t>elc_spv_067</t>
-  </si>
-  <si>
-    <t>rez_spv_068</t>
-  </si>
-  <si>
-    <t>elc_spv_068</t>
-  </si>
-  <si>
-    <t>rez_spv_069</t>
-  </si>
-  <si>
-    <t>elc_spv_069</t>
-  </si>
-  <si>
-    <t>rez_spv_070</t>
-  </si>
-  <si>
-    <t>elc_spv_070</t>
-  </si>
-  <si>
-    <t>rez_spv_071</t>
-  </si>
-  <si>
-    <t>elc_spv_071</t>
-  </si>
-  <si>
-    <t>rez_spv_072</t>
-  </si>
-  <si>
-    <t>elc_spv_072</t>
-  </si>
-  <si>
-    <t>rez_spv_073</t>
-  </si>
-  <si>
-    <t>elc_spv_073</t>
-  </si>
-  <si>
-    <t>rez_spv_074</t>
-  </si>
-  <si>
-    <t>elc_spv_074</t>
-  </si>
-  <si>
-    <t>rez_won_001</t>
-  </si>
-  <si>
-    <t>elc_won_001</t>
-  </si>
-  <si>
-    <t>rez_won_002</t>
-  </si>
-  <si>
-    <t>elc_won_002</t>
-  </si>
-  <si>
-    <t>rez_won_003</t>
-  </si>
-  <si>
-    <t>elc_won_003</t>
-  </si>
-  <si>
-    <t>rez_won_004</t>
-  </si>
-  <si>
-    <t>elc_won_004</t>
-  </si>
-  <si>
-    <t>rez_won_005</t>
-  </si>
-  <si>
-    <t>elc_won_005</t>
-  </si>
-  <si>
-    <t>rez_won_006</t>
-  </si>
-  <si>
-    <t>elc_won_006</t>
-  </si>
-  <si>
-    <t>rez_won_007</t>
-  </si>
-  <si>
-    <t>elc_won_007</t>
-  </si>
-  <si>
-    <t>rez_won_008</t>
-  </si>
-  <si>
-    <t>elc_won_008</t>
-  </si>
-  <si>
-    <t>rez_won_009</t>
-  </si>
-  <si>
-    <t>elc_won_009</t>
-  </si>
-  <si>
-    <t>rez_won_010</t>
-  </si>
-  <si>
-    <t>elc_won_010</t>
-  </si>
-  <si>
-    <t>rez_won_011</t>
-  </si>
-  <si>
-    <t>elc_won_011</t>
-  </si>
-  <si>
-    <t>rez_won_012</t>
-  </si>
-  <si>
-    <t>elc_won_012</t>
-  </si>
-  <si>
-    <t>rez_won_013</t>
-  </si>
-  <si>
-    <t>elc_won_013</t>
-  </si>
-  <si>
-    <t>rez_won_014</t>
-  </si>
-  <si>
-    <t>elc_won_014</t>
-  </si>
-  <si>
-    <t>rez_won_015</t>
-  </si>
-  <si>
-    <t>elc_won_015</t>
-  </si>
-  <si>
-    <t>rez_won_016</t>
-  </si>
-  <si>
-    <t>elc_won_016</t>
-  </si>
-  <si>
-    <t>rez_won_017</t>
-  </si>
-  <si>
-    <t>elc_won_017</t>
-  </si>
-  <si>
-    <t>rez_won_018</t>
-  </si>
-  <si>
-    <t>elc_won_018</t>
-  </si>
-  <si>
-    <t>rez_won_019</t>
-  </si>
-  <si>
-    <t>elc_won_019</t>
-  </si>
-  <si>
-    <t>rez_won_020</t>
-  </si>
-  <si>
-    <t>elc_won_020</t>
-  </si>
-  <si>
-    <t>rez_won_021</t>
-  </si>
-  <si>
-    <t>elc_won_021</t>
-  </si>
-  <si>
-    <t>rez_won_022</t>
-  </si>
-  <si>
-    <t>elc_won_022</t>
-  </si>
-  <si>
-    <t>rez_won_023</t>
-  </si>
-  <si>
-    <t>elc_won_023</t>
-  </si>
-  <si>
-    <t>rez_won_024</t>
-  </si>
-  <si>
-    <t>elc_won_024</t>
-  </si>
-  <si>
-    <t>rez_won_025</t>
-  </si>
-  <si>
-    <t>elc_won_025</t>
-  </si>
-  <si>
-    <t>rez_won_026</t>
-  </si>
-  <si>
-    <t>elc_won_026</t>
-  </si>
-  <si>
-    <t>rez_won_027</t>
-  </si>
-  <si>
-    <t>elc_won_027</t>
-  </si>
-  <si>
-    <t>rez_won_028</t>
-  </si>
-  <si>
-    <t>elc_won_028</t>
-  </si>
-  <si>
-    <t>rez_won_029</t>
-  </si>
-  <si>
-    <t>elc_won_029</t>
-  </si>
-  <si>
-    <t>rez_won_030</t>
-  </si>
-  <si>
-    <t>elc_won_030</t>
-  </si>
-  <si>
-    <t>rez_won_031</t>
-  </si>
-  <si>
-    <t>elc_won_031</t>
-  </si>
-  <si>
-    <t>rez_won_032</t>
-  </si>
-  <si>
-    <t>elc_won_032</t>
-  </si>
-  <si>
-    <t>rez_won_033</t>
-  </si>
-  <si>
-    <t>elc_won_033</t>
-  </si>
-  <si>
-    <t>rez_won_034</t>
-  </si>
-  <si>
-    <t>elc_won_034</t>
-  </si>
-  <si>
-    <t>rez_won_035</t>
-  </si>
-  <si>
-    <t>elc_won_035</t>
-  </si>
-  <si>
-    <t>rez_won_036</t>
-  </si>
-  <si>
-    <t>elc_won_036</t>
-  </si>
-  <si>
-    <t>rez_wof_001</t>
-  </si>
-  <si>
-    <t>elc_wof_001</t>
-  </si>
-  <si>
-    <t>rez_wof_002</t>
-  </si>
-  <si>
-    <t>elc_wof_002</t>
-  </si>
-  <si>
-    <t>rez_wof_003</t>
-  </si>
-  <si>
-    <t>elc_wof_003</t>
-  </si>
-  <si>
-    <t>rez_wof_004</t>
-  </si>
-  <si>
-    <t>elc_wof_004</t>
-  </si>
-  <si>
-    <t>rez_wof_005</t>
-  </si>
-  <si>
-    <t>elc_wof_005</t>
-  </si>
-  <si>
-    <t>rez_wof_006</t>
-  </si>
-  <si>
-    <t>elc_wof_006</t>
-  </si>
-  <si>
-    <t>rez_wof_007</t>
-  </si>
-  <si>
-    <t>elc_wof_007</t>
-  </si>
-  <si>
-    <t>rez_wof_008</t>
-  </si>
-  <si>
-    <t>elc_wof_008</t>
-  </si>
-  <si>
-    <t>rez_wof_009</t>
-  </si>
-  <si>
-    <t>elc_wof_009</t>
-  </si>
-  <si>
-    <t>rez_wof_010</t>
-  </si>
-  <si>
-    <t>elc_wof_010</t>
-  </si>
-  <si>
-    <t>rez_wof_011</t>
-  </si>
-  <si>
-    <t>elc_wof_011</t>
-  </si>
-  <si>
-    <t>rez_wof_012</t>
-  </si>
-  <si>
-    <t>elc_wof_012</t>
-  </si>
-  <si>
-    <t>rez_wof_013</t>
-  </si>
-  <si>
-    <t>elc_wof_013</t>
-  </si>
-  <si>
-    <t>rez_wof_014</t>
-  </si>
-  <si>
-    <t>elc_wof_014</t>
-  </si>
-  <si>
-    <t>rez_wof_015</t>
-  </si>
-  <si>
-    <t>elc_wof_015</t>
-  </si>
-  <si>
-    <t>rez_wof_016</t>
-  </si>
-  <si>
-    <t>elc_wof_016</t>
-  </si>
-  <si>
-    <t>rez_wof_017</t>
-  </si>
-  <si>
-    <t>elc_wof_017</t>
-  </si>
-  <si>
-    <t>rez_wof_018</t>
-  </si>
-  <si>
-    <t>elc_wof_018</t>
-  </si>
-  <si>
-    <t>rez_wof_019</t>
-  </si>
-  <si>
-    <t>elc_wof_019</t>
-  </si>
-  <si>
-    <t>rez_wof_020</t>
-  </si>
-  <si>
-    <t>elc_wof_020</t>
-  </si>
-  <si>
-    <t>rez_wof_021</t>
-  </si>
-  <si>
-    <t>elc_wof_021</t>
-  </si>
-  <si>
-    <t>rez_wof_022</t>
-  </si>
-  <si>
-    <t>elc_wof_022</t>
-  </si>
-  <si>
-    <t>rez_wof_023</t>
-  </si>
-  <si>
-    <t>elc_wof_023</t>
-  </si>
-  <si>
-    <t>rez_wof_024</t>
-  </si>
-  <si>
-    <t>elc_wof_024</t>
-  </si>
-  <si>
-    <t>rez_wof_025</t>
-  </si>
-  <si>
-    <t>elc_wof_025</t>
-  </si>
-  <si>
-    <t>rez_wof_026</t>
-  </si>
-  <si>
-    <t>elc_wof_026</t>
-  </si>
-  <si>
-    <t>rez_wof_027</t>
-  </si>
-  <si>
-    <t>elc_wof_027</t>
-  </si>
-  <si>
-    <t>rez_wof_028</t>
-  </si>
-  <si>
-    <t>elc_wof_028</t>
-  </si>
-  <si>
-    <t>rez_wof_029</t>
-  </si>
-  <si>
-    <t>elc_wof_029</t>
-  </si>
-  <si>
-    <t>rez_wof_030</t>
-  </si>
-  <si>
-    <t>elc_wof_030</t>
-  </si>
-  <si>
-    <t>rez_wof_031</t>
-  </si>
-  <si>
-    <t>elc_wof_031</t>
-  </si>
-  <si>
-    <t>rez_wof_032</t>
-  </si>
-  <si>
-    <t>elc_wof_032</t>
-  </si>
-  <si>
-    <t>rez_wof_033</t>
-  </si>
-  <si>
-    <t>elc_wof_033</t>
-  </si>
-  <si>
-    <t>rez_wof_034</t>
-  </si>
-  <si>
-    <t>elc_wof_034</t>
-  </si>
-  <si>
-    <t>rez_wof_035</t>
-  </si>
-  <si>
-    <t>elc_wof_035</t>
+    <t>p_w161960924-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w161960924-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w161960933-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w161960933-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w161965853-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w161965853-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w166633831-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w166633831-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w169444592-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w169444592-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w261185002-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w261185002-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w264410236-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w264410236-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w264550744-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w264550744-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w265318414-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w265318414-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w265568001-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w265568001-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w267626657-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w267626657-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w271376037-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w271376037-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w310695690-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w310695690-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w310958602-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w310958602-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w314452486-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w314452486-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w337039411-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w337039411-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w340205049-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w340205049-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w340978681-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w340978681-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w398909640-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w398909640-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w399038181-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w399038181-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w399100034-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w399100034-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w399100035-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w399100035-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w469888049-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w469888049-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w527900241-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w527900241-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w528189342-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w528189342-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w544403426-230_IDN</t>
+  </si>
+  <si>
+    <t>e_w544403426-230_IDN*</t>
+  </si>
+  <si>
+    <t>p_w544403431-230_IDN</t>
+  </si>
+  <si>
+    <t>e_w544403431-230_IDN*</t>
+  </si>
+  <si>
+    <t>p_w562061281-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w562061281-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w604684007-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w604684007-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w610198177-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w610198177-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w614955990-230_IDN</t>
+  </si>
+  <si>
+    <t>e_w614955990-230_IDN*</t>
+  </si>
+  <si>
+    <t>p_w614955993-230_IDN</t>
+  </si>
+  <si>
+    <t>e_w614955993-230_IDN*</t>
+  </si>
+  <si>
+    <t>p_w615581232-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w615581232-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w615581242-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w615581242-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w615581270-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w615581270-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w629512849-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w629512849-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w662591948-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w662591948-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w689263666-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w689263666-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w721674155-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w721674155-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w721685825-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w721685825-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w736595653-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w736595653-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w753733608-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w753733608-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w754073846-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w754073846-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w754096394-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w754096394-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w754178666-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w754178666-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w754178667-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w754178667-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w759130125-230_IDN</t>
+  </si>
+  <si>
+    <t>e_w759130125-230_IDN*</t>
+  </si>
+  <si>
+    <t>p_w769617021-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w769617021-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w841499143-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w841499143-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w926254403-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w926254403-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w928220391-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w928220391-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w928928133-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w928928133-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w930719092-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w930719092-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w931931121-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w931931121-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w931931133-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w931931133-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w939542521-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w939542521-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w943539373-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w943539373-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w946191122-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w946191122-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w960747902-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w960747902-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w960747936-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w960747936-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w966209515-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w966209515-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w1013653012-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w1013653012-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w1186182648-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w1186182648-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w1193553154-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w1193553154-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w1308433899-500_IDN</t>
+  </si>
+  <si>
+    <t>e_w1308433899-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w1312287191-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w1312287191-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w1316786278-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w1316786278-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w1316876158-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w1316876158-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID36-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID36-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID11-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID11-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID26-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID26-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID13-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID13-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID22-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID22-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID38-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID38-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID34-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID34-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID1-275_IDN</t>
+  </si>
+  <si>
+    <t>e_ID1-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_w943539373-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w943539373-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID31-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID31-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_w736595653-275_IDN</t>
+  </si>
+  <si>
+    <t>e_w736595653-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID4-275_IDN</t>
+  </si>
+  <si>
+    <t>e_ID4-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID5-275_IDN</t>
+  </si>
+  <si>
+    <t>e_ID5-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID6-275_IDN</t>
+  </si>
+  <si>
+    <t>e_ID6-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID7-275_IDN</t>
+  </si>
+  <si>
+    <t>e_ID7-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID12-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID12-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID28-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID28-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID27-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID27-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID25-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID25-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID33-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID33-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID37-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID37-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID10-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID10-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID16-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID16-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID8-275_IDN</t>
+  </si>
+  <si>
+    <t>e_ID8-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID14-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID14-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID18-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID18-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID21-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID21-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID20-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID20-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID24-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID24-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID2-275_IDN</t>
+  </si>
+  <si>
+    <t>e_ID2-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID9-230_IDN</t>
+  </si>
+  <si>
+    <t>e_ID9-230_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID30-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID30-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID3-275_IDN</t>
+  </si>
+  <si>
+    <t>e_ID3-275_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID23-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID23-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID29-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID29-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID35-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID35-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID19-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID19-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID17-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID17-500_IDN*</t>
+  </si>
+  <si>
+    <t>p_ID15-500_IDN</t>
+  </si>
+  <si>
+    <t>e_ID15-500_IDN*</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_001</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_001</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_002</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_002</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_003</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_003</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_004</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_004</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_005</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_005</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_006</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_006</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_007</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_007</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_008</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_008</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_009</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_009</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_010</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_010</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_011</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_011</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_012</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_012</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_013</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_013</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_014</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_014</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_015</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_015</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_016</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_016</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_017</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_017</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_018</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_018</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_019</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_019</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_020</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_020</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_021</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_021</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_022</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_022</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_023</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_023</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_024</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_024</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_025</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_025</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_026</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_026</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_027</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_027</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_028</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_028</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_029</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_029</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_030</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_030</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_031</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_031</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_032</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_032</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_033</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_033</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_034</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_034</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_035</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_035</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_036</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_036</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_037</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_037</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_038</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_038</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_039</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_039</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_040</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_040</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_041</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_041</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_042</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_042</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_043</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_043</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_044</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_044</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_045</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_045</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_046</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_046</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_047</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_047</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_048</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_048</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_049</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_049</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_050</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_050</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_051</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_051</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_052</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_052</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_053</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_053</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_054</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_054</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_055</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_055</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_056</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_056</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_057</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_057</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_058</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_058</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_059</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_059</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_060</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_060</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_061</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_061</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_062</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_062</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_063</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_063</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_064</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_064</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_065</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_065</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_066</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_066</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_067</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_067</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_068</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_068</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_069</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_069</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_070</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_070</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_071</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_071</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_072</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_072</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_073</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_073</t>
+  </si>
+  <si>
+    <t>rez_spv_IDN_074</t>
+  </si>
+  <si>
+    <t>elc_spv_IDN_074</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_001</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_001</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_002</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_002</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_003</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_003</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_004</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_004</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_005</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_005</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_006</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_006</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_007</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_007</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_008</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_008</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_009</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_009</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_010</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_010</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_011</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_011</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_012</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_012</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_013</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_013</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_014</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_014</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_015</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_015</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_016</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_016</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_017</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_017</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_018</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_018</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_019</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_019</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_020</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_020</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_021</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_021</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_022</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_022</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_023</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_023</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_024</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_024</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_025</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_025</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_026</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_026</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_027</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_027</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_028</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_028</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_029</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_029</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_030</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_030</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_031</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_031</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_032</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_032</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_033</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_033</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_034</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_034</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_035</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_035</t>
+  </si>
+  <si>
+    <t>rez_won_IDN_036</t>
+  </si>
+  <si>
+    <t>elc_won_IDN_036</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_001</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_001</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_002</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_002</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_003</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_003</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_004</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_004</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_005</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_005</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_006</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_006</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_007</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_007</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_008</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_008</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_009</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_009</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_010</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_010</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_011</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_011</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_012</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_012</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_013</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_013</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_014</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_014</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_015</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_015</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_016</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_016</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_017</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_017</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_018</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_018</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_019</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_019</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_020</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_020</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_021</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_021</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_022</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_022</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_023</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_023</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_024</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_024</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_025</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_025</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_026</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_026</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_027</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_027</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_028</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_028</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_029</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_029</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_030</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_030</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_031</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_031</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_032</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_032</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_033</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_033</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_034</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_034</t>
+  </si>
+  <si>
+    <t>rez_wof_IDN_035</t>
+  </si>
+  <si>
+    <t>elc_wof_IDN_035</t>
   </si>
 </sst>
 </file>
@@ -2693,8 +2705,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D193CE7F-0CD9-482D-AB9E-7E8C12A7423E}">
-  <dimension ref="B9:E261"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDD32239-0BA1-444F-A5AC-5817064E1D31}">
+  <dimension ref="B9:E263"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="9" spans="2:5" x14ac:dyDescent="0.45">
@@ -6227,6 +6239,34 @@
         <v>605</v>
       </c>
       <c r="E261" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="262" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B262" t="s">
+        <v>606</v>
+      </c>
+      <c r="C262" t="s">
+        <v>607</v>
+      </c>
+      <c r="D262" t="s">
+        <v>607</v>
+      </c>
+      <c r="E262" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="263" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B263" t="s">
+        <v>608</v>
+      </c>
+      <c r="C263" t="s">
+        <v>609</v>
+      </c>
+      <c r="D263" t="s">
+        <v>609</v>
+      </c>
+      <c r="E263" t="s">
         <v>105</v>
       </c>
     </row>

</xml_diff>